<commit_message>
v0.2.2-alpha - Big update
- updated bunch of mods
- removed CraftTweaker and addons for testing purpose
- removed matmos because of high cpu and ram consumption, generally it's not needed at all
- added LeafCulling for testing purpose, cheking performance impact
- migrated from unofficial ver of EC to actual one
- added several backport mods:
-- backhand
-- campfirebackport
</commit_message>
<xml_diff>
--- a/list of all ids.xlsx
+++ b/list of all ids.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AVM\Desktop\foxies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C80E6AC9-A1C2-4768-AE71-27838B5359A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9792AFFD-2561-4AB1-8FA8-2DD2F092A2FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="225" yWindow="840" windowWidth="27405" windowHeight="14760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Измерения" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="358">
   <si>
     <t>Название измерения</t>
   </si>
@@ -1096,6 +1096,12 @@
   </si>
   <si>
     <t>Evil</t>
+  </si>
+  <si>
+    <t>WorldEngine biome</t>
+  </si>
+  <si>
+    <t>ASJCore</t>
   </si>
 </sst>
 </file>
@@ -2762,7 +2768,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:I146"/>
+  <dimension ref="A1:I147"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.42578125" style="5" customWidth="1"/>
@@ -3028,95 +3034,101 @@
       <c r="D23" s="25"/>
     </row>
     <row r="24" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
-        <v>7</v>
+      <c r="A24" s="11" t="s">
+        <v>353</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" s="6">
-        <v>126</v>
+        <v>337</v>
+      </c>
+      <c r="C24" s="19">
+        <v>106</v>
+      </c>
+      <c r="D24" s="27">
+        <v>180</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25" s="6">
-        <v>127</v>
+      <c r="A25" s="11" t="s">
+        <v>353</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>338</v>
+      </c>
+      <c r="C25" s="19">
+        <v>107</v>
+      </c>
+      <c r="D25" s="27">
+        <v>174</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>230</v>
+        <v>339</v>
       </c>
       <c r="C26" s="19">
-        <v>128</v>
+        <v>108</v>
       </c>
       <c r="D26" s="27">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>237</v>
+        <v>340</v>
       </c>
       <c r="C27" s="19">
-        <v>135</v>
+        <v>109</v>
       </c>
       <c r="D27" s="27">
-        <v>190</v>
+        <v>172</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>238</v>
+        <v>341</v>
       </c>
       <c r="C28" s="19">
-        <v>136</v>
+        <v>110</v>
       </c>
       <c r="D28" s="27">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>239</v>
+        <v>342</v>
       </c>
       <c r="C29" s="19">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="D29" s="27">
-        <v>203</v>
+        <v>178</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>240</v>
+        <v>343</v>
       </c>
       <c r="C30" s="19">
-        <v>138</v>
+        <v>112</v>
       </c>
       <c r="D30" s="27">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="22"/>
@@ -3126,170 +3138,166 @@
     </row>
     <row r="31" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>241</v>
+        <v>344</v>
       </c>
       <c r="C31" s="19">
-        <v>139</v>
+        <v>113</v>
       </c>
       <c r="D31" s="11">
-        <v>196</v>
+        <v>184</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>243</v>
+        <v>345</v>
       </c>
       <c r="C32" s="19">
-        <v>141</v>
+        <v>114</v>
       </c>
       <c r="D32" s="11">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>244</v>
+        <v>346</v>
       </c>
       <c r="C33" s="19">
-        <v>142</v>
+        <v>115</v>
       </c>
       <c r="D33" s="11">
-        <v>177</v>
+        <v>185</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>245</v>
+        <v>347</v>
       </c>
       <c r="C34" s="19">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="D34" s="11">
-        <v>210</v>
+        <v>183</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>246</v>
+        <v>348</v>
       </c>
       <c r="C35" s="19">
-        <v>144</v>
+        <v>117</v>
       </c>
       <c r="D35" s="11">
-        <v>204</v>
+        <v>176</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>247</v>
+        <v>349</v>
       </c>
       <c r="C36" s="19">
-        <v>145</v>
+        <v>118</v>
       </c>
       <c r="D36" s="11">
-        <v>213</v>
+        <v>171</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>248</v>
+        <v>350</v>
       </c>
       <c r="C37" s="19">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="D37" s="11">
-        <v>212</v>
+        <v>181</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>249</v>
+        <v>351</v>
       </c>
       <c r="C38" s="19">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="D38" s="11">
-        <v>211</v>
+        <v>175</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>250</v>
+        <v>352</v>
       </c>
       <c r="C39" s="19">
-        <v>148</v>
+        <v>121</v>
       </c>
       <c r="D39" s="11">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="11" t="s">
-        <v>229</v>
+      <c r="A40" s="6" t="s">
+        <v>7</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>252</v>
-      </c>
-      <c r="C40" s="19">
-        <v>150</v>
-      </c>
-      <c r="D40" s="11">
-        <v>185</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="C40" s="6">
+        <v>126</v>
+      </c>
+      <c r="D40" s="25"/>
     </row>
     <row r="41" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="B41" s="11" t="s">
-        <v>254</v>
-      </c>
-      <c r="C41" s="19">
-        <v>152</v>
-      </c>
-      <c r="D41" s="11">
-        <v>178</v>
-      </c>
+      <c r="A41" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" s="6">
+        <v>127</v>
+      </c>
+      <c r="D41" s="25"/>
     </row>
     <row r="42" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>229</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>255</v>
+        <v>230</v>
       </c>
       <c r="C42" s="19">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="D42" s="11">
-        <v>148</v>
+        <v>170</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3297,13 +3305,13 @@
         <v>229</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
       <c r="C43" s="19">
-        <v>154</v>
+        <v>135</v>
       </c>
       <c r="D43" s="11">
-        <v>153</v>
+        <v>190</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3311,13 +3319,13 @@
         <v>229</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>257</v>
+        <v>238</v>
       </c>
       <c r="C44" s="19">
-        <v>155</v>
+        <v>136</v>
       </c>
       <c r="D44" s="11">
-        <v>200</v>
+        <v>182</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3325,13 +3333,13 @@
         <v>229</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>261</v>
+        <v>239</v>
       </c>
       <c r="C45" s="19">
-        <v>159</v>
+        <v>137</v>
       </c>
       <c r="D45" s="11">
-        <v>194</v>
+        <v>203</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3339,13 +3347,13 @@
         <v>229</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>264</v>
+        <v>240</v>
       </c>
       <c r="C46" s="19">
-        <v>177</v>
+        <v>138</v>
       </c>
       <c r="D46" s="11">
-        <v>172</v>
+        <v>150</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3353,13 +3361,13 @@
         <v>229</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>270</v>
+        <v>241</v>
       </c>
       <c r="C47" s="19">
-        <v>168</v>
+        <v>139</v>
       </c>
       <c r="D47" s="11">
-        <v>186</v>
+        <v>196</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3367,13 +3375,13 @@
         <v>229</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>271</v>
+        <v>243</v>
       </c>
       <c r="C48" s="19">
-        <v>169</v>
+        <v>141</v>
       </c>
       <c r="D48" s="11">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3381,13 +3389,13 @@
         <v>229</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>272</v>
+        <v>244</v>
       </c>
       <c r="C49" s="19">
-        <v>170</v>
+        <v>142</v>
       </c>
       <c r="D49" s="11">
-        <v>169</v>
+        <v>177</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3395,13 +3403,13 @@
         <v>229</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>273</v>
+        <v>245</v>
       </c>
       <c r="C50" s="19">
-        <v>171</v>
+        <v>143</v>
       </c>
       <c r="D50" s="11">
-        <v>187</v>
+        <v>210</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3409,13 +3417,13 @@
         <v>229</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>274</v>
+        <v>246</v>
       </c>
       <c r="C51" s="19">
-        <v>172</v>
+        <v>144</v>
       </c>
       <c r="D51" s="11">
-        <v>188</v>
+        <v>204</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3423,13 +3431,13 @@
         <v>229</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>275</v>
+        <v>247</v>
       </c>
       <c r="C52" s="19">
-        <v>173</v>
+        <v>145</v>
       </c>
       <c r="D52" s="11">
-        <v>152</v>
+        <v>213</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3437,13 +3445,13 @@
         <v>229</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>276</v>
+        <v>248</v>
       </c>
       <c r="C53" s="19">
-        <v>174</v>
+        <v>146</v>
       </c>
       <c r="D53" s="11">
-        <v>191</v>
+        <v>212</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3451,13 +3459,13 @@
         <v>229</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>277</v>
+        <v>249</v>
       </c>
       <c r="C54" s="19">
-        <v>175</v>
+        <v>147</v>
       </c>
       <c r="D54" s="11">
-        <v>192</v>
+        <v>211</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3465,105 +3473,114 @@
         <v>229</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>278</v>
+        <v>250</v>
       </c>
       <c r="C55" s="19">
-        <v>176</v>
+        <v>148</v>
       </c>
       <c r="D55" s="11">
-        <v>145</v>
+        <v>174</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
-        <v>25</v>
+        <v>229</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C56" s="6">
-        <v>192</v>
-      </c>
-      <c r="D56" s="25"/>
+        <v>252</v>
+      </c>
+      <c r="C56" s="19">
+        <v>150</v>
+      </c>
+      <c r="D56" s="11">
+        <v>185</v>
+      </c>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
-        <v>25</v>
+        <v>229</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C57" s="6">
-        <v>193</v>
-      </c>
-      <c r="D57" s="25"/>
+        <v>254</v>
+      </c>
+      <c r="C57" s="19">
+        <v>152</v>
+      </c>
+      <c r="D57" s="11">
+        <v>178</v>
+      </c>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
-        <v>25</v>
+        <v>229</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C58" s="6">
-        <v>194</v>
-      </c>
-      <c r="D58" s="25"/>
+        <v>255</v>
+      </c>
+      <c r="C58" s="19">
+        <v>153</v>
+      </c>
+      <c r="D58" s="11">
+        <v>148</v>
+      </c>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
-        <v>25</v>
+        <v>229</v>
       </c>
       <c r="B59" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C59" s="11">
-        <v>195</v>
-      </c>
-      <c r="D59" s="25"/>
+        <v>256</v>
+      </c>
+      <c r="C59" s="19">
+        <v>154</v>
+      </c>
+      <c r="D59" s="11">
+        <v>153</v>
+      </c>
       <c r="E59" s="23"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>224</v>
+        <v>257</v>
       </c>
       <c r="C60" s="19">
-        <v>220</v>
-      </c>
-      <c r="D60" s="24">
-        <v>102</v>
-      </c>
-      <c r="E60" s="22"/>
+        <v>155</v>
+      </c>
+      <c r="D60" s="11">
+        <v>200</v>
+      </c>
+      <c r="E60" s="23"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="11" t="s">
         <v>229</v>
       </c>
       <c r="B61" s="11" t="s">
-        <v>231</v>
+        <v>261</v>
       </c>
       <c r="C61" s="19">
-        <v>201</v>
+        <v>159</v>
       </c>
       <c r="D61" s="11">
-        <v>146</v>
-      </c>
+        <v>194</v>
+      </c>
+      <c r="E61" s="22"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
         <v>229</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>233</v>
+        <v>270</v>
       </c>
       <c r="C62" s="19">
-        <v>202</v>
+        <v>168</v>
       </c>
       <c r="D62" s="11">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3571,13 +3588,13 @@
         <v>229</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="C63" s="19">
-        <v>203</v>
+        <v>169</v>
       </c>
       <c r="D63" s="11">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3585,13 +3602,13 @@
         <v>229</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="C64" s="19">
-        <v>204</v>
+        <v>170</v>
       </c>
       <c r="D64" s="11">
-        <v>176</v>
+        <v>169</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3599,13 +3616,13 @@
         <v>229</v>
       </c>
       <c r="B65" s="11" t="s">
-        <v>253</v>
+        <v>273</v>
       </c>
       <c r="C65" s="19">
-        <v>205</v>
+        <v>171</v>
       </c>
       <c r="D65" s="11">
-        <v>195</v>
+        <v>187</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3613,13 +3630,13 @@
         <v>229</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>258</v>
+        <v>274</v>
       </c>
       <c r="C66" s="19">
-        <v>206</v>
+        <v>172</v>
       </c>
       <c r="D66" s="11">
-        <v>199</v>
+        <v>188</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3627,13 +3644,13 @@
         <v>229</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="C67" s="19">
-        <v>207</v>
+        <v>173</v>
       </c>
       <c r="D67" s="11">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3641,13 +3658,13 @@
         <v>229</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="C68" s="19">
-        <v>208</v>
+        <v>174</v>
       </c>
       <c r="D68" s="11">
-        <v>147</v>
+        <v>191</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3655,13 +3672,13 @@
         <v>229</v>
       </c>
       <c r="B69" s="11" t="s">
-        <v>266</v>
+        <v>277</v>
       </c>
       <c r="C69" s="19">
-        <v>209</v>
+        <v>175</v>
       </c>
       <c r="D69" s="11">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3669,13 +3686,13 @@
         <v>229</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="C70" s="19">
-        <v>210</v>
+        <v>176</v>
       </c>
       <c r="D70" s="11">
-        <v>201</v>
+        <v>145</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3683,84 +3700,76 @@
         <v>229</v>
       </c>
       <c r="B71" s="11" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C71" s="19">
-        <v>211</v>
+        <v>177</v>
       </c>
       <c r="D71" s="11">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
-        <v>229</v>
+        <v>25</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>269</v>
-      </c>
-      <c r="C72" s="19">
-        <v>212</v>
-      </c>
-      <c r="D72" s="11">
-        <v>202</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="C72" s="6">
+        <v>192</v>
+      </c>
+      <c r="D72" s="25"/>
     </row>
     <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
-        <v>229</v>
+        <v>25</v>
       </c>
       <c r="B73" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="C73" s="19">
-        <v>213</v>
-      </c>
-      <c r="D73" s="11">
-        <v>159</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="C73" s="6">
+        <v>193</v>
+      </c>
+      <c r="D73" s="25"/>
     </row>
     <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
-        <v>229</v>
+        <v>25</v>
       </c>
       <c r="B74" s="11" t="s">
-        <v>234</v>
-      </c>
-      <c r="C74" s="19">
-        <v>214</v>
-      </c>
-      <c r="D74" s="11">
-        <v>183</v>
-      </c>
-      <c r="E74" s="23"/>
+        <v>26</v>
+      </c>
+      <c r="C74" s="6">
+        <v>194</v>
+      </c>
+      <c r="D74" s="25"/>
     </row>
     <row r="75" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
-        <v>229</v>
+        <v>25</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>235</v>
-      </c>
-      <c r="C75" s="19">
-        <v>215</v>
-      </c>
-      <c r="D75" s="11">
-        <v>171</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="C75" s="11">
+        <v>195</v>
+      </c>
+      <c r="D75" s="25"/>
+      <c r="E75" s="23"/>
     </row>
     <row r="76" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
         <v>229</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="C76" s="19">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="D76" s="11">
-        <v>181</v>
+        <v>146</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3768,13 +3777,13 @@
         <v>229</v>
       </c>
       <c r="B77" s="11" t="s">
-        <v>259</v>
+        <v>233</v>
       </c>
       <c r="C77" s="19">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="D77" s="11">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3782,13 +3791,13 @@
         <v>229</v>
       </c>
       <c r="B78" s="11" t="s">
-        <v>260</v>
+        <v>242</v>
       </c>
       <c r="C78" s="19">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="D78" s="11">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3796,237 +3805,237 @@
         <v>229</v>
       </c>
       <c r="B79" s="11" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="C79" s="19">
-        <v>219</v>
+        <v>204</v>
       </c>
       <c r="D79" s="11">
-        <v>168</v>
+        <v>176</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B80" s="11" t="s">
-        <v>312</v>
+        <v>253</v>
       </c>
       <c r="C80" s="19">
-        <v>245</v>
+        <v>205</v>
       </c>
       <c r="D80" s="11">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B81" s="11" t="s">
-        <v>313</v>
+        <v>258</v>
       </c>
       <c r="C81" s="19">
-        <v>246</v>
+        <v>206</v>
       </c>
       <c r="D81" s="11">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="82" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>314</v>
+        <v>263</v>
       </c>
       <c r="C82" s="19">
-        <v>247</v>
+        <v>207</v>
       </c>
       <c r="D82" s="11">
-        <v>202</v>
+        <v>154</v>
       </c>
     </row>
     <row r="83" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B83" s="11" t="s">
-        <v>315</v>
+        <v>265</v>
       </c>
       <c r="C83" s="19">
-        <v>248</v>
+        <v>208</v>
       </c>
       <c r="D83" s="11">
-        <v>203</v>
+        <v>147</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>316</v>
+        <v>266</v>
       </c>
       <c r="C84" s="19">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="D84" s="11">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B85" s="11" t="s">
-        <v>317</v>
+        <v>267</v>
       </c>
       <c r="C85" s="19">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="D85" s="11">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>318</v>
+        <v>268</v>
       </c>
       <c r="C86" s="19">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="D86" s="11">
-        <v>206</v>
+        <v>173</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B87" s="11" t="s">
-        <v>319</v>
+        <v>269</v>
       </c>
       <c r="C87" s="19">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="D87" s="11">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>320</v>
+        <v>232</v>
       </c>
       <c r="C88" s="19">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="D88" s="11">
-        <v>208</v>
+        <v>159</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>321</v>
+        <v>234</v>
       </c>
       <c r="C89" s="19">
-        <v>229</v>
+        <v>214</v>
       </c>
       <c r="D89" s="11">
-        <v>209</v>
+        <v>183</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>322</v>
+        <v>235</v>
       </c>
       <c r="C90" s="19">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="D90" s="11">
-        <v>210</v>
+        <v>171</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B91" s="11" t="s">
-        <v>323</v>
+        <v>236</v>
       </c>
       <c r="C91" s="19">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="D91" s="11">
-        <v>211</v>
+        <v>181</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B92" s="11" t="s">
-        <v>324</v>
+        <v>259</v>
       </c>
       <c r="C92" s="19">
-        <v>232</v>
+        <v>217</v>
       </c>
       <c r="D92" s="11">
-        <v>212</v>
+        <v>179</v>
       </c>
     </row>
     <row r="93" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B93" s="11" t="s">
-        <v>325</v>
+        <v>260</v>
       </c>
       <c r="C93" s="19">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="D93" s="11">
-        <v>213</v>
+        <v>193</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="11" t="s">
-        <v>311</v>
+        <v>229</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>326</v>
+        <v>262</v>
       </c>
       <c r="C94" s="19">
-        <v>234</v>
+        <v>219</v>
       </c>
       <c r="D94" s="11">
-        <v>214</v>
+        <v>168</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="11" t="s">
-        <v>311</v>
+        <v>223</v>
       </c>
       <c r="B95" s="11" t="s">
-        <v>327</v>
+        <v>224</v>
       </c>
       <c r="C95" s="19">
-        <v>235</v>
-      </c>
-      <c r="D95" s="11">
-        <v>215</v>
+        <v>220</v>
+      </c>
+      <c r="D95" s="24">
+        <v>102</v>
       </c>
     </row>
     <row r="96" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -4034,13 +4043,13 @@
         <v>311</v>
       </c>
       <c r="B96" s="11" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="C96" s="19">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="D96" s="11">
-        <v>216</v>
+        <v>204</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -4048,13 +4057,13 @@
         <v>311</v>
       </c>
       <c r="B97" s="11" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="C97" s="19">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="D97" s="11">
-        <v>217</v>
+        <v>205</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -4062,13 +4071,13 @@
         <v>311</v>
       </c>
       <c r="B98" s="11" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="C98" s="19">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="D98" s="11">
-        <v>218</v>
+        <v>206</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -4076,13 +4085,13 @@
         <v>311</v>
       </c>
       <c r="B99" s="11" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="C99" s="19">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="D99" s="11">
-        <v>219</v>
+        <v>207</v>
       </c>
     </row>
     <row r="100" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -4090,13 +4099,13 @@
         <v>311</v>
       </c>
       <c r="B100" s="11" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="C100" s="19">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="D100" s="11">
-        <v>220</v>
+        <v>208</v>
       </c>
     </row>
     <row r="101" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -4104,13 +4113,13 @@
         <v>311</v>
       </c>
       <c r="B101" s="11" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="C101" s="19">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="D101" s="11">
-        <v>221</v>
+        <v>209</v>
       </c>
     </row>
     <row r="102" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -4118,13 +4127,13 @@
         <v>311</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
       <c r="C102" s="19">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="D102" s="11">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="103" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -4132,13 +4141,13 @@
         <v>311</v>
       </c>
       <c r="B103" s="11" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
       <c r="C103" s="19">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="D103" s="11">
-        <v>223</v>
+        <v>211</v>
       </c>
     </row>
     <row r="104" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -4146,243 +4155,252 @@
         <v>311</v>
       </c>
       <c r="B104" s="11" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="C104" s="19">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="D104" s="11">
-        <v>224</v>
+        <v>212</v>
       </c>
     </row>
     <row r="105" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B105" s="11" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="C105" s="19">
-        <v>106</v>
-      </c>
-      <c r="D105" s="33">
-        <v>180</v>
+        <v>233</v>
+      </c>
+      <c r="D105" s="11">
+        <v>213</v>
       </c>
     </row>
     <row r="106" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B106" s="11" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="C106" s="19">
-        <v>107</v>
+        <v>234</v>
       </c>
       <c r="D106" s="33">
-        <v>174</v>
+        <v>214</v>
       </c>
     </row>
     <row r="107" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B107" s="11" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="C107" s="19">
-        <v>108</v>
+        <v>235</v>
       </c>
       <c r="D107" s="33">
-        <v>173</v>
+        <v>215</v>
       </c>
     </row>
     <row r="108" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B108" s="11" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="C108" s="19">
-        <v>109</v>
+        <v>236</v>
       </c>
       <c r="D108" s="33">
-        <v>172</v>
+        <v>216</v>
       </c>
     </row>
     <row r="109" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B109" s="11" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
       <c r="C109" s="19">
-        <v>110</v>
+        <v>237</v>
       </c>
       <c r="D109" s="33">
-        <v>179</v>
+        <v>217</v>
       </c>
     </row>
     <row r="110" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B110" s="11" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="C110" s="19">
-        <v>111</v>
+        <v>238</v>
       </c>
       <c r="D110" s="33">
-        <v>178</v>
+        <v>218</v>
       </c>
     </row>
     <row r="111" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B111" s="11" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="C111" s="19">
-        <v>112</v>
+        <v>239</v>
       </c>
       <c r="D111" s="33">
-        <v>170</v>
+        <v>219</v>
       </c>
     </row>
     <row r="112" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B112" s="11" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="C112" s="19">
-        <v>113</v>
+        <v>240</v>
       </c>
       <c r="D112" s="33">
-        <v>184</v>
+        <v>220</v>
       </c>
     </row>
     <row r="113" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
       <c r="C113" s="19">
-        <v>114</v>
+        <v>241</v>
       </c>
       <c r="D113" s="33">
-        <v>182</v>
+        <v>221</v>
       </c>
     </row>
     <row r="114" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B114" s="11" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="C114" s="19">
-        <v>115</v>
+        <v>242</v>
       </c>
       <c r="D114" s="33">
-        <v>185</v>
+        <v>222</v>
       </c>
     </row>
     <row r="115" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B115" s="11" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
       <c r="C115" s="19">
-        <v>116</v>
+        <v>243</v>
       </c>
       <c r="D115" s="33">
-        <v>183</v>
+        <v>223</v>
       </c>
     </row>
     <row r="116" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B116" s="11" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="C116" s="19">
-        <v>117</v>
+        <v>244</v>
       </c>
       <c r="D116" s="33">
-        <v>176</v>
+        <v>224</v>
       </c>
     </row>
     <row r="117" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B117" s="11" t="s">
-        <v>349</v>
+        <v>312</v>
       </c>
       <c r="C117" s="19">
-        <v>118</v>
+        <v>245</v>
       </c>
       <c r="D117" s="33">
-        <v>171</v>
+        <v>200</v>
       </c>
     </row>
     <row r="118" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B118" s="11" t="s">
-        <v>350</v>
+        <v>313</v>
       </c>
       <c r="C118" s="19">
-        <v>119</v>
+        <v>246</v>
       </c>
       <c r="D118" s="33">
-        <v>181</v>
+        <v>201</v>
       </c>
     </row>
     <row r="119" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B119" s="11" t="s">
-        <v>351</v>
+        <v>314</v>
       </c>
       <c r="C119" s="19">
-        <v>120</v>
+        <v>247</v>
       </c>
       <c r="D119" s="33">
-        <v>175</v>
+        <v>202</v>
       </c>
     </row>
     <row r="120" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="11" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="B120" s="11" t="s">
-        <v>352</v>
+        <v>315</v>
       </c>
       <c r="C120" s="19">
-        <v>121</v>
+        <v>248</v>
       </c>
       <c r="D120" s="33">
-        <v>177</v>
+        <v>203</v>
       </c>
     </row>
     <row r="121" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="11"/>
-      <c r="B121" s="11"/>
-      <c r="C121" s="19"/>
+      <c r="A121" s="11" t="s">
+        <v>357</v>
+      </c>
+      <c r="B121" s="11" t="s">
+        <v>356</v>
+      </c>
+      <c r="C121" s="19">
+        <v>60</v>
+      </c>
+      <c r="D121" s="33">
+        <v>150</v>
+      </c>
     </row>
     <row r="122" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="11"/>
@@ -4399,7 +4417,11 @@
       <c r="B124" s="11"/>
       <c r="C124" s="19"/>
     </row>
-    <row r="125" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="11"/>
+      <c r="B125" s="11"/>
+      <c r="C125" s="19"/>
+    </row>
     <row r="126" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="127" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="128" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4421,9 +4443,10 @@
     <row r="144" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="145" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="146" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="147" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E146">
-    <sortCondition ref="C2:C146"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D147">
+    <sortCondition ref="C1:C147"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>